<commit_message>
Added TC_16 to TC_20
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PractoLogin_TestData.xlsx
+++ b/src/test/resources/testData/PractoLogin_TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497837\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497845\IdeaProjects\Finding-Hospitals\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80C3D0A-E738-48EF-8789-7626062A9916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3D5432-A6CA-47F3-8BB1-D4AECAE55884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="770" yWindow="1810" windowWidth="8940" windowHeight="8180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -36,34 +36,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
-    <t>Mobile Number/Email</t>
+    <t>Abcd</t>
   </si>
   <si>
-    <t>Password</t>
+    <t>CCTSS</t>
   </si>
   <si>
-    <t>9092270105</t>
+    <t>abcd@gmail.com</t>
   </si>
   <si>
-    <t>Yp22330011@</t>
+    <t>abcd</t>
   </si>
   <si>
-    <t>WrongPass123</t>
-  </si>
-  <si>
-    <t>abc123</t>
-  </si>
-  <si>
-    <t>@@@###</t>
+    <t>abcdmail:com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,9 +66,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -85,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -93,32 +96,22 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -419,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.90625" customWidth="1"/>
@@ -434,42 +427,54 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>9876543210</v>
+      </c>
+      <c r="B3" s="1">
+        <v>987654321</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="mailto:abcd@gmail.com" xr:uid="{ED5EF57D-7B10-4416-BE57-2461389D0979}"/>
+    <hyperlink ref="B4" r:id="rId2" display="mailto:abcd@gmail.com" xr:uid="{49A42C1C-F911-4C7C-AB9D-0A0EA3F937B8}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added ScreenShot function in TestCases
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PractoLogin_TestData.xlsx
+++ b/src/test/resources/testData/PractoLogin_TestData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497845\IdeaProjects\Finding-Hospitals\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3D5432-A6CA-47F3-8BB1-D4AECAE55884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5955D9F2-7B5B-4827-B626-A3348807491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="770" yWindow="1810" windowWidth="8940" windowHeight="8180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
+    <sheet name="PatientData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Abcd</t>
   </si>
@@ -51,6 +52,12 @@
   </si>
   <si>
     <t>abcdmail:com</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>john213gmail</t>
   </si>
 </sst>
 </file>
@@ -101,12 +108,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -477,4 +487,37 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030A4899-4444-41BA-8FBE-480FA936B1BC}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>1234567890</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Modified LoginData in xlsx
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PractoLogin_TestData.xlsx
+++ b/src/test/resources/testData/PractoLogin_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497845\IdeaProjects\Finding-Hospitals\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5955D9F2-7B5B-4827-B626-A3348807491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC30A9D-0E3E-41D3-817C-9063CAC1290C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -37,17 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
-  <si>
-    <t>Abcd</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>CCTSS</t>
   </si>
   <si>
-    <t>abcd@gmail.com</t>
-  </si>
-  <si>
     <t>abcd</t>
   </si>
   <si>
@@ -58,6 +52,15 @@
   </si>
   <si>
     <t>john213gmail</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>CTS</t>
+  </si>
+  <si>
+    <t>john123@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -434,18 +437,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -458,10 +461,10 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -482,7 +485,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" display="mailto:abcd@gmail.com" xr:uid="{ED5EF57D-7B10-4416-BE57-2461389D0979}"/>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{ED5EF57D-7B10-4416-BE57-2461389D0979}"/>
     <hyperlink ref="B4" r:id="rId2" display="mailto:abcd@gmail.com" xr:uid="{49A42C1C-F911-4C7C-AB9D-0A0EA3F937B8}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -499,7 +502,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -514,7 +517,7 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>